<commit_message>
DBDP-62: fix DHP-SMR record_id collision via content discriminator (budget_sub_activity_title); add record_id uniqueness post-run assertion; regenerate parquet + Excel
</commit_message>
<xml_diff>
--- a/output/ODBA_FY2027_Budget_Report.xlsx
+++ b/output/ODBA_FY2027_Budget_Report.xlsx
@@ -31632,7 +31632,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>009d82a7350d</t>
+          <t>25e91742f948</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
@@ -31713,7 +31713,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>69cc198f960b</t>
+          <t>d2877e003eea</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
@@ -31794,7 +31794,7 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>bf95da34ddce</t>
+          <t>19432d9279fd</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
@@ -31875,7 +31875,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>a737cbb92826</t>
+          <t>e5fedd0242c3</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
@@ -31956,7 +31956,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>b3dd06311c3c</t>
+          <t>83768482b37e</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
@@ -32037,7 +32037,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>789b08a6287c</t>
+          <t>7a772c7fdb18</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
@@ -32118,7 +32118,7 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>a7363f5539ee</t>
+          <t>4b2a918f4d28</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
@@ -32199,7 +32199,7 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>2cb1fe9c8c9e</t>
+          <t>5b82d1421e0b</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
@@ -32280,7 +32280,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>f24fbb9a4e0c</t>
+          <t>178c89e74537</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
@@ -32361,7 +32361,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>3a0de3337138</t>
+          <t>44149e3bd9ab</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
@@ -32442,7 +32442,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>60702e374585</t>
+          <t>360e58fa8495</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
@@ -32523,7 +32523,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>3348ccb81131</t>
+          <t>f6358361d471</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
@@ -32604,7 +32604,7 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>60702e374585</t>
+          <t>c38d2a59bb0e</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
@@ -32685,7 +32685,7 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>374ca6e2e5f0</t>
+          <t>4c1296b2e30b</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
@@ -32766,7 +32766,7 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>bc2e02f09bd0</t>
+          <t>8bdb2dfd4b71</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
@@ -32847,7 +32847,7 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>f1cf24ba207a</t>
+          <t>085fb7ba1f6f</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
@@ -32928,7 +32928,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>94b2b8409cd3</t>
+          <t>80d4d484197d</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
@@ -33009,7 +33009,7 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>fd7b808a493f</t>
+          <t>d4fec4192ed0</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
@@ -33090,7 +33090,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>0be05415ce33</t>
+          <t>bd1e602c8627</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
@@ -33171,7 +33171,7 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>f24fbb9a4e0c</t>
+          <t>75ae49a7ee51</t>
         </is>
       </c>
       <c r="B24" s="7" t="n">
@@ -33252,7 +33252,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>0be05415ce33</t>
+          <t>ebcda3bb5269</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
@@ -33333,7 +33333,7 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>94b2b8409cd3</t>
+          <t>3aea291c4af0</t>
         </is>
       </c>
       <c r="B26" s="7" t="n">
@@ -33414,7 +33414,7 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>9c384dc239fb</t>
+          <t>a2463703b797</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
@@ -33495,7 +33495,7 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>60702e374585</t>
+          <t>95056abc6cf1</t>
         </is>
       </c>
       <c r="B28" s="7" t="n">
@@ -33576,7 +33576,7 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>bc2e02f09bd0</t>
+          <t>fe8e1974f906</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
@@ -33657,7 +33657,7 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>0be05415ce33</t>
+          <t>83532785f053</t>
         </is>
       </c>
       <c r="B30" s="7" t="n">
@@ -33738,7 +33738,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>12be44519554</t>
+          <t>19105792f64b</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
@@ -33819,7 +33819,7 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>94b2b8409cd3</t>
+          <t>616243d7a314</t>
         </is>
       </c>
       <c r="B32" s="7" t="n">
@@ -33900,7 +33900,7 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>fd7b808a493f</t>
+          <t>b2eac4993fce</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
@@ -34548,7 +34548,7 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>128247e20bc1</t>
+          <t>b34c2490273a</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
@@ -34629,7 +34629,7 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>d34905558852</t>
+          <t>5bcee9e050fc</t>
         </is>
       </c>
       <c r="B42" s="7" t="n">
@@ -34710,7 +34710,7 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>7d0788a3224f</t>
+          <t>e10f5a5fe2e6</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
@@ -34791,7 +34791,7 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>7d0788a3224f</t>
+          <t>3ef27032b7c5</t>
         </is>
       </c>
       <c r="B44" s="7" t="n">
@@ -34872,7 +34872,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>0f27ceee5b47</t>
+          <t>311e8c072ccb</t>
         </is>
       </c>
       <c r="B45" s="4" t="n">
@@ -34953,7 +34953,7 @@
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>0914f31e4786</t>
+          <t>f5f381d9b9a1</t>
         </is>
       </c>
       <c r="B46" s="7" t="n">
@@ -35034,7 +35034,7 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>7d0788a3224f</t>
+          <t>7e78f788258e</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
@@ -35115,7 +35115,7 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>7d0788a3224f</t>
+          <t>580392dc8f38</t>
         </is>
       </c>
       <c r="B48" s="7" t="n">
@@ -35196,7 +35196,7 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>a800ad241033</t>
+          <t>a4dd7e1747d2</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">

</xml_diff>